<commit_message>
FiRe LEAGUE Buenos Aires
</commit_message>
<xml_diff>
--- a/file/old.xlsx
+++ b/file/old.xlsx
@@ -469,7 +469,7 @@
         <v>1155.8269573717953</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -484,13 +484,13 @@
         <v>AM</v>
       </c>
       <c r="K2" t="str">
-        <v>none</v>
+        <v>major</v>
       </c>
       <c r="L2">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="M2" t="str">
-        <v>2026-07-05T04:08:18.328Z</v>
+        <v>2026-07-07T13:04:25.872Z</v>
       </c>
       <c r="N2" t="str">
         <v/>
@@ -1408,7 +1408,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Take Flyte</v>
+        <v>Entropiq</v>
       </c>
       <c r="B20">
         <v>3</v>
@@ -1420,7 +1420,7 @@
         <v>2</v>
       </c>
       <c r="E20">
-        <v>1015.6724304703677</v>
+        <v>1016.3039403297893</v>
       </c>
       <c r="F20">
         <v>0</v>
@@ -1444,7 +1444,7 @@
         <v>0</v>
       </c>
       <c r="M20" t="str">
-        <v>2026-07-05T04:05:23.392Z</v>
+        <v>2026-07-07T04:08:42.949Z</v>
       </c>
       <c r="N20" t="str">
         <v/>
@@ -1461,19 +1461,19 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>The Huns</v>
+        <v>Take Flyte</v>
       </c>
       <c r="B21">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E21">
-        <v>1015</v>
+        <v>1015.6724304703677</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -1497,7 +1497,7 @@
         <v>0</v>
       </c>
       <c r="M21" t="str">
-        <v>2026-02-18T21:21:06.168Z</v>
+        <v>2026-07-05T04:05:23.392Z</v>
       </c>
       <c r="N21" t="str">
         <v/>
@@ -1514,19 +1514,19 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Onyx Ravens</v>
+        <v>The Huns</v>
       </c>
       <c r="B22">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E22">
-        <v>1014.9877256835035</v>
+        <v>1015</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -1550,7 +1550,7 @@
         <v>0</v>
       </c>
       <c r="M22" t="str">
-        <v>2026-03-21T04:32:33.790Z</v>
+        <v>2026-02-18T21:21:06.168Z</v>
       </c>
       <c r="N22" t="str">
         <v/>
@@ -1567,19 +1567,19 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>TYLOO</v>
+        <v>Onyx Ravens</v>
       </c>
       <c r="B23">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C23">
         <v>0</v>
       </c>
       <c r="D23">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E23">
-        <v>1014.128742285643</v>
+        <v>1014.9877256835035</v>
       </c>
       <c r="F23">
         <v>0</v>
@@ -1594,7 +1594,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J23" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>AM</v>
       </c>
       <c r="K23" t="str">
         <v>none</v>
@@ -1603,7 +1603,7 @@
         <v>0</v>
       </c>
       <c r="M23" t="str">
-        <v>2026-02-19T22:09:16.526Z</v>
+        <v>2026-03-21T04:32:33.790Z</v>
       </c>
       <c r="N23" t="str">
         <v/>
@@ -1620,19 +1620,19 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>OG</v>
+        <v>Counter Logic</v>
       </c>
       <c r="B24">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E24">
-        <v>1013.5266895185538</v>
+        <v>1014.6510123894305</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -1647,7 +1647,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J24" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K24" t="str">
         <v>none</v>
@@ -1656,7 +1656,7 @@
         <v>0</v>
       </c>
       <c r="M24" t="str">
-        <v>2026-02-19T22:09:03.691Z</v>
+        <v>2026-07-07T04:08:50.601Z</v>
       </c>
       <c r="N24" t="str">
         <v/>
@@ -1673,19 +1673,19 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Into the Beach</v>
+        <v>TYLOO</v>
       </c>
       <c r="B25">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E25">
-        <v>1011.823225766436</v>
+        <v>1014.128742285643</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1700,7 +1700,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J25" t="str">
-        <v>AM</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K25" t="str">
         <v>none</v>
@@ -1709,7 +1709,7 @@
         <v>0</v>
       </c>
       <c r="M25" t="str">
-        <v>2026-07-05T04:07:15.376Z</v>
+        <v>2026-02-19T22:09:16.526Z</v>
       </c>
       <c r="N25" t="str">
         <v/>
@@ -1726,19 +1726,19 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>BESTIA</v>
+        <v>OG</v>
       </c>
       <c r="B26">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C26">
         <v>0</v>
       </c>
       <c r="D26">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E26">
-        <v>1005.0046329623956</v>
+        <v>1013.5266895185538</v>
       </c>
       <c r="F26">
         <v>0</v>
@@ -1753,7 +1753,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J26" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K26" t="str">
         <v>none</v>
@@ -1762,7 +1762,7 @@
         <v>0</v>
       </c>
       <c r="M26" t="str">
-        <v>2026-02-28T06:29:16.752Z</v>
+        <v>2026-02-19T22:09:03.691Z</v>
       </c>
       <c r="N26" t="str">
         <v/>
@@ -1779,19 +1779,19 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>G2</v>
+        <v>Into the Beach</v>
       </c>
       <c r="B27">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E27">
-        <v>1002.6421965170028</v>
+        <v>1011.823225766436</v>
       </c>
       <c r="F27">
         <v>0</v>
@@ -1806,7 +1806,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J27" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K27" t="str">
         <v>none</v>
@@ -1815,7 +1815,7 @@
         <v>0</v>
       </c>
       <c r="M27" t="str">
-        <v>2026-02-28T06:28:17.433Z</v>
+        <v>2026-07-05T04:07:15.376Z</v>
       </c>
       <c r="N27" t="str">
         <v/>
@@ -1832,19 +1832,19 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>FURIA</v>
+        <v>BESTIA</v>
       </c>
       <c r="B28">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E28">
-        <v>1001.9019624181617</v>
+        <v>1005.0046329623956</v>
       </c>
       <c r="F28">
         <v>0</v>
@@ -1868,7 +1868,7 @@
         <v>0</v>
       </c>
       <c r="M28" t="str">
-        <v>2026-06-26T13:19:31.639Z</v>
+        <v>2026-02-28T06:29:16.752Z</v>
       </c>
       <c r="N28" t="str">
         <v/>
@@ -1885,19 +1885,19 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Mythic</v>
+        <v>G2</v>
       </c>
       <c r="B29">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E29">
-        <v>1000.942849124707</v>
+        <v>1002.6421965170028</v>
       </c>
       <c r="F29">
         <v>0</v>
@@ -1912,7 +1912,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J29" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K29" t="str">
         <v>none</v>
@@ -1921,7 +1921,7 @@
         <v>0</v>
       </c>
       <c r="M29" t="str">
-        <v>2026-07-05T04:05:49.346Z</v>
+        <v>2026-02-28T06:28:17.433Z</v>
       </c>
       <c r="N29" t="str">
         <v/>
@@ -1938,19 +1938,19 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>hoorai</v>
+        <v>FURIA</v>
       </c>
       <c r="B30">
         <v>4</v>
       </c>
       <c r="C30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30">
         <v>4</v>
       </c>
       <c r="E30">
-        <v>1000.4888979238718</v>
+        <v>1001.9019624181617</v>
       </c>
       <c r="F30">
         <v>0</v>
@@ -1965,7 +1965,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J30" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K30" t="str">
         <v>none</v>
@@ -1974,7 +1974,7 @@
         <v>0</v>
       </c>
       <c r="M30" t="str">
-        <v>2026-02-28T06:28:25.661Z</v>
+        <v>2026-06-26T13:19:31.639Z</v>
       </c>
       <c r="N30" t="str">
         <v/>
@@ -1991,19 +1991,19 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>00 Nation</v>
+        <v>Mythic</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D31">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E31">
-        <v>1000</v>
+        <v>1000.942849124707</v>
       </c>
       <c r="F31">
         <v>0</v>
@@ -2018,7 +2018,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J31" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K31" t="str">
         <v>none</v>
@@ -2027,7 +2027,7 @@
         <v>0</v>
       </c>
       <c r="M31" t="str">
-        <v/>
+        <v>2026-07-05T04:05:49.346Z</v>
       </c>
       <c r="N31" t="str">
         <v/>
@@ -2044,19 +2044,19 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>100 Thieves</v>
+        <v>hoorai</v>
       </c>
       <c r="B32">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C32">
         <v>0</v>
       </c>
       <c r="D32">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E32">
-        <v>1000</v>
+        <v>1000.4888979238718</v>
       </c>
       <c r="F32">
         <v>0</v>
@@ -2080,7 +2080,7 @@
         <v>0</v>
       </c>
       <c r="M32" t="str">
-        <v/>
+        <v>2026-02-28T06:28:25.661Z</v>
       </c>
       <c r="N32" t="str">
         <v/>
@@ -2097,7 +2097,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Astana Dragons</v>
+        <v>00 Nation</v>
       </c>
       <c r="B33">
         <v>0</v>
@@ -2150,7 +2150,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Astralis Talent</v>
+        <v>100 Thieves</v>
       </c>
       <c r="B34">
         <v>0</v>
@@ -2203,7 +2203,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Avangar</v>
+        <v>Astana Dragons</v>
       </c>
       <c r="B35">
         <v>0</v>
@@ -2230,7 +2230,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J35" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>EU</v>
       </c>
       <c r="K35" t="str">
         <v>none</v>
@@ -2256,7 +2256,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>BIG Academy</v>
+        <v>Astralis Talent</v>
       </c>
       <c r="B36">
         <v>0</v>
@@ -2309,7 +2309,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Bravado</v>
+        <v>Avangar</v>
       </c>
       <c r="B37">
         <v>0</v>
@@ -2362,7 +2362,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Copenhagen Wolves</v>
+        <v>BIG Academy</v>
       </c>
       <c r="B38">
         <v>0</v>
@@ -2415,7 +2415,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Counter Logic</v>
+        <v>Bravado</v>
       </c>
       <c r="B39">
         <v>0</v>
@@ -2442,7 +2442,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J39" t="str">
-        <v>AM</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K39" t="str">
         <v>none</v>
@@ -2468,7 +2468,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ENCE Academy</v>
+        <v>Copenhagen Wolves</v>
       </c>
       <c r="B40">
         <v>0</v>
@@ -2521,7 +2521,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ESC</v>
+        <v>ENCE Academy</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -2574,7 +2574,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Flash</v>
+        <v>ESC</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -2627,7 +2627,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>FLuffy Gangsters</v>
+        <v>Flash</v>
       </c>
       <c r="B43">
         <v>0</v>
@@ -2680,7 +2680,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>FlyQuest RED</v>
+        <v>FLuffy Gangsters</v>
       </c>
       <c r="B44">
         <v>0</v>
@@ -2733,7 +2733,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Fnatic</v>
+        <v>FlyQuest RED</v>
       </c>
       <c r="B45">
         <v>0</v>
@@ -2786,7 +2786,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>FORZE</v>
+        <v>Fnatic</v>
       </c>
       <c r="B46">
         <v>0</v>
@@ -2813,7 +2813,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J46" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>EU</v>
       </c>
       <c r="K46" t="str">
         <v>none</v>
@@ -2839,7 +2839,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Gambit</v>
+        <v>FORZE</v>
       </c>
       <c r="B47">
         <v>0</v>
@@ -2866,7 +2866,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J47" t="str">
-        <v>EU</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K47" t="str">
         <v>none</v>
@@ -2892,7 +2892,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>GATERON</v>
+        <v>Gambit</v>
       </c>
       <c r="B48">
         <v>0</v>
@@ -2919,7 +2919,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J48" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>EU</v>
       </c>
       <c r="K48" t="str">
         <v>none</v>
@@ -2945,7 +2945,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>GhoulsW</v>
+        <v>GATERON</v>
       </c>
       <c r="B49">
         <v>0</v>
@@ -2972,7 +2972,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J49" t="str">
-        <v>EU</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K49" t="str">
         <v>none</v>
@@ -2998,7 +2998,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>HAVU</v>
+        <v>GhoulsW</v>
       </c>
       <c r="B50">
         <v>0</v>
@@ -3051,7 +3051,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Heroic Academy</v>
+        <v>HAVU</v>
       </c>
       <c r="B51">
         <v>0</v>
@@ -3104,7 +3104,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Hesta</v>
+        <v>Heroic Academy</v>
       </c>
       <c r="B52">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Kinguin</v>
+        <v>Hesta</v>
       </c>
       <c r="B53">
         <v>0</v>
@@ -3210,7 +3210,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>kONO</v>
+        <v>Kinguin</v>
       </c>
       <c r="B54">
         <v>0</v>
@@ -3237,7 +3237,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J54" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>EU</v>
       </c>
       <c r="K54" t="str">
         <v>none</v>
@@ -3263,7 +3263,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>LGB</v>
+        <v>kONO</v>
       </c>
       <c r="B55">
         <v>0</v>
@@ -3316,7 +3316,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>MAD Lions</v>
+        <v>LGB</v>
       </c>
       <c r="B56">
         <v>0</v>
@@ -3343,7 +3343,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J56" t="str">
-        <v>EU</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K56" t="str">
         <v>none</v>
@@ -3369,7 +3369,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Misfits</v>
+        <v>MAD Lions</v>
       </c>
       <c r="B57">
         <v>0</v>
@@ -3422,7 +3422,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>mousesports</v>
+        <v>Misfits</v>
       </c>
       <c r="B58">
         <v>0</v>
@@ -3475,7 +3475,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>MOUZ NXT</v>
+        <v>mousesports</v>
       </c>
       <c r="B59">
         <v>0</v>
@@ -3528,7 +3528,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Movistar KOI</v>
+        <v>MOUZ NXT</v>
       </c>
       <c r="B60">
         <v>0</v>
@@ -3581,7 +3581,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>NIP Impact</v>
+        <v>Movistar KOI</v>
       </c>
       <c r="B61">
         <v>0</v>
@@ -3634,7 +3634,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Nordix</v>
+        <v>NIP Impact</v>
       </c>
       <c r="B62">
         <v>0</v>
@@ -3687,7 +3687,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>NOVAQ</v>
+        <v>Nordix</v>
       </c>
       <c r="B63">
         <v>0</v>
@@ -3740,7 +3740,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>paiN Academy</v>
+        <v>NOVAQ</v>
       </c>
       <c r="B64">
         <v>0</v>
@@ -3767,7 +3767,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J64" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K64" t="str">
         <v>none</v>
@@ -4111,7 +4111,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Sprout</v>
+        <v>Tsunami</v>
       </c>
       <c r="B71">
         <v>0</v>
@@ -4138,7 +4138,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J71" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K71" t="str">
         <v>none</v>
@@ -4164,7 +4164,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Tsunami</v>
+        <v>VeryGames</v>
       </c>
       <c r="B72">
         <v>0</v>
@@ -4217,7 +4217,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>VeryGames</v>
+        <v>Vox Eminor</v>
       </c>
       <c r="B73">
         <v>0</v>
@@ -4270,7 +4270,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Vox Eminor</v>
+        <v>Wildcard Academy</v>
       </c>
       <c r="B74">
         <v>0</v>
@@ -4323,7 +4323,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Wildcard Academy</v>
+        <v>Lux Tenebris</v>
       </c>
       <c r="B75">
         <v>0</v>
@@ -4350,7 +4350,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J75" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K75" t="str">
         <v>none</v>
@@ -4376,19 +4376,19 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Lux Tenebris</v>
+        <v>Spirit Academy</v>
       </c>
       <c r="B76">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C76">
         <v>0</v>
       </c>
       <c r="D76">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E76">
-        <v>1000</v>
+        <v>999.7251809772306</v>
       </c>
       <c r="F76">
         <v>0</v>
@@ -4403,7 +4403,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J76" t="str">
-        <v>AM</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K76" t="str">
         <v>none</v>
@@ -4412,7 +4412,7 @@
         <v>0</v>
       </c>
       <c r="M76" t="str">
-        <v/>
+        <v>2026-02-19T02:49:35.870Z</v>
       </c>
       <c r="N76" t="str">
         <v/>
@@ -4429,7 +4429,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Spirit Academy</v>
+        <v>True Rippers</v>
       </c>
       <c r="B77">
         <v>2</v>
@@ -4456,7 +4456,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J77" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>EU</v>
       </c>
       <c r="K77" t="str">
         <v>none</v>
@@ -4465,7 +4465,7 @@
         <v>0</v>
       </c>
       <c r="M77" t="str">
-        <v>2026-02-19T02:49:35.870Z</v>
+        <v>2026-02-19T02:47:38.886Z</v>
       </c>
       <c r="N77" t="str">
         <v/>
@@ -4482,7 +4482,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>True Rippers</v>
+        <v>FaZe</v>
       </c>
       <c r="B78">
         <v>2</v>
@@ -4518,7 +4518,7 @@
         <v>0</v>
       </c>
       <c r="M78" t="str">
-        <v>2026-02-19T02:47:38.886Z</v>
+        <v>2026-02-19T02:36:39.932Z</v>
       </c>
       <c r="N78" t="str">
         <v/>
@@ -4535,7 +4535,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>FaZe</v>
+        <v>iBUYPOWER</v>
       </c>
       <c r="B79">
         <v>2</v>
@@ -4571,7 +4571,7 @@
         <v>0</v>
       </c>
       <c r="M79" t="str">
-        <v>2026-02-19T02:36:39.932Z</v>
+        <v>2026-02-19T02:36:34.302Z</v>
       </c>
       <c r="N79" t="str">
         <v/>
@@ -4588,7 +4588,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>iBUYPOWER</v>
+        <v>GODSENT</v>
       </c>
       <c r="B80">
         <v>2</v>
@@ -4615,7 +4615,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J80" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K80" t="str">
         <v>none</v>
@@ -4624,7 +4624,7 @@
         <v>0</v>
       </c>
       <c r="M80" t="str">
-        <v>2026-02-19T02:36:34.302Z</v>
+        <v>2026-02-19T01:39:32.364Z</v>
       </c>
       <c r="N80" t="str">
         <v/>
@@ -4641,7 +4641,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>GODSENT</v>
+        <v>M80</v>
       </c>
       <c r="B81">
         <v>2</v>
@@ -4653,7 +4653,7 @@
         <v>2</v>
       </c>
       <c r="E81">
-        <v>999.7251809772306</v>
+        <v>999.672340544519</v>
       </c>
       <c r="F81">
         <v>0</v>
@@ -4677,7 +4677,7 @@
         <v>0</v>
       </c>
       <c r="M81" t="str">
-        <v>2026-02-19T01:39:32.364Z</v>
+        <v>2026-02-19T01:45:45.455Z</v>
       </c>
       <c r="N81" t="str">
         <v/>
@@ -4694,19 +4694,19 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>M80</v>
+        <v>Chinggis Warriors</v>
       </c>
       <c r="B82">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C82">
         <v>0</v>
       </c>
       <c r="D82">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E82">
-        <v>999.672340544519</v>
+        <v>999.4408194717619</v>
       </c>
       <c r="F82">
         <v>0</v>
@@ -4721,7 +4721,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J82" t="str">
-        <v>AM</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K82" t="str">
         <v>none</v>
@@ -4730,7 +4730,7 @@
         <v>0</v>
       </c>
       <c r="M82" t="str">
-        <v>2026-02-19T01:45:45.455Z</v>
+        <v>2026-02-19T22:08:18.806Z</v>
       </c>
       <c r="N82" t="str">
         <v/>
@@ -4747,7 +4747,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Chinggis Warriors</v>
+        <v>Orbit</v>
       </c>
       <c r="B83">
         <v>3</v>
@@ -4759,7 +4759,7 @@
         <v>3</v>
       </c>
       <c r="E83">
-        <v>999.4408194717619</v>
+        <v>999.4186945376644</v>
       </c>
       <c r="F83">
         <v>0</v>
@@ -4774,7 +4774,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J83" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>EU</v>
       </c>
       <c r="K83" t="str">
         <v>none</v>
@@ -4783,7 +4783,7 @@
         <v>0</v>
       </c>
       <c r="M83" t="str">
-        <v>2026-02-19T22:08:18.806Z</v>
+        <v>2026-02-19T22:08:33.993Z</v>
       </c>
       <c r="N83" t="str">
         <v/>
@@ -4800,19 +4800,19 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>Orbit</v>
+        <v>Alliance</v>
       </c>
       <c r="B84">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C84">
         <v>0</v>
       </c>
       <c r="D84">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E84">
-        <v>999.4186945376644</v>
+        <v>999.4088515186523</v>
       </c>
       <c r="F84">
         <v>0</v>
@@ -4836,7 +4836,7 @@
         <v>0</v>
       </c>
       <c r="M84" t="str">
-        <v>2026-02-19T22:08:33.993Z</v>
+        <v>2026-02-19T02:51:22.336Z</v>
       </c>
       <c r="N84" t="str">
         <v/>
@@ -4853,7 +4853,7 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Alliance</v>
+        <v>Homyno</v>
       </c>
       <c r="B85">
         <v>2</v>
@@ -4880,7 +4880,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J85" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K85" t="str">
         <v>none</v>
@@ -4889,7 +4889,7 @@
         <v>0</v>
       </c>
       <c r="M85" t="str">
-        <v>2026-02-19T02:51:22.336Z</v>
+        <v>2026-02-19T02:51:16.607Z</v>
       </c>
       <c r="N85" t="str">
         <v/>
@@ -4906,7 +4906,7 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Homyno</v>
+        <v>MenaceGG</v>
       </c>
       <c r="B86">
         <v>2</v>
@@ -4933,7 +4933,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J86" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K86" t="str">
         <v>none</v>
@@ -4942,7 +4942,7 @@
         <v>0</v>
       </c>
       <c r="M86" t="str">
-        <v>2026-02-19T02:51:16.607Z</v>
+        <v>2026-02-19T02:49:44.165Z</v>
       </c>
       <c r="N86" t="str">
         <v/>
@@ -4959,7 +4959,7 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>MenaceGG</v>
+        <v>Solid</v>
       </c>
       <c r="B87">
         <v>2</v>
@@ -4986,7 +4986,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J87" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K87" t="str">
         <v>none</v>
@@ -4995,7 +4995,7 @@
         <v>0</v>
       </c>
       <c r="M87" t="str">
-        <v>2026-02-19T02:49:44.165Z</v>
+        <v>2026-02-19T02:47:50.233Z</v>
       </c>
       <c r="N87" t="str">
         <v/>
@@ -5012,7 +5012,7 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Solid</v>
+        <v>ENCE</v>
       </c>
       <c r="B88">
         <v>2</v>
@@ -5039,7 +5039,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J88" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K88" t="str">
         <v>none</v>
@@ -5048,7 +5048,7 @@
         <v>0</v>
       </c>
       <c r="M88" t="str">
-        <v>2026-02-19T02:47:50.233Z</v>
+        <v>2026-02-19T02:34:19.604Z</v>
       </c>
       <c r="N88" t="str">
         <v/>
@@ -5065,7 +5065,7 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>ENCE</v>
+        <v>Nexus</v>
       </c>
       <c r="B89">
         <v>2</v>
@@ -5101,7 +5101,7 @@
         <v>0</v>
       </c>
       <c r="M89" t="str">
-        <v>2026-02-19T02:34:19.604Z</v>
+        <v>2026-02-19T02:34:13.227Z</v>
       </c>
       <c r="N89" t="str">
         <v/>
@@ -5118,7 +5118,7 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Nexus</v>
+        <v>MIBR</v>
       </c>
       <c r="B90">
         <v>2</v>
@@ -5145,7 +5145,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J90" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K90" t="str">
         <v>none</v>
@@ -5154,7 +5154,7 @@
         <v>0</v>
       </c>
       <c r="M90" t="str">
-        <v>2026-02-19T02:34:13.227Z</v>
+        <v>2026-02-19T01:39:50.018Z</v>
       </c>
       <c r="N90" t="str">
         <v/>
@@ -5171,7 +5171,7 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>MIBR</v>
+        <v>Wizards</v>
       </c>
       <c r="B91">
         <v>2</v>
@@ -5183,7 +5183,7 @@
         <v>2</v>
       </c>
       <c r="E91">
-        <v>999.4088515186523</v>
+        <v>999.4062521695108</v>
       </c>
       <c r="F91">
         <v>0</v>
@@ -5207,7 +5207,7 @@
         <v>0</v>
       </c>
       <c r="M91" t="str">
-        <v>2026-02-19T01:39:50.018Z</v>
+        <v>2026-02-19T01:45:38.841Z</v>
       </c>
       <c r="N91" t="str">
         <v/>
@@ -5224,19 +5224,19 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Wizards</v>
+        <v>RED Canids</v>
       </c>
       <c r="B92">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C92">
         <v>0</v>
       </c>
       <c r="D92">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E92">
-        <v>999.4062521695108</v>
+        <v>999.3397745397444</v>
       </c>
       <c r="F92">
         <v>0</v>
@@ -5260,7 +5260,7 @@
         <v>0</v>
       </c>
       <c r="M92" t="str">
-        <v>2026-02-19T01:45:38.841Z</v>
+        <v>2026-02-19T22:08:44.661Z</v>
       </c>
       <c r="N92" t="str">
         <v/>
@@ -5277,19 +5277,19 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>RED Canids</v>
+        <v>Rebels</v>
       </c>
       <c r="B93">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C93">
         <v>0</v>
       </c>
       <c r="D93">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E93">
-        <v>999.3397745397444</v>
+        <v>999.3232682842747</v>
       </c>
       <c r="F93">
         <v>0</v>
@@ -5304,7 +5304,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J93" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K93" t="str">
         <v>none</v>
@@ -5313,7 +5313,7 @@
         <v>0</v>
       </c>
       <c r="M93" t="str">
-        <v>2026-02-19T22:08:44.661Z</v>
+        <v>2026-02-28T06:28:39.554Z</v>
       </c>
       <c r="N93" t="str">
         <v/>
@@ -5330,19 +5330,19 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Rebels</v>
+        <v>Legacy</v>
       </c>
       <c r="B94">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C94">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D94">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E94">
-        <v>999.3232682842747</v>
+        <v>991.3908681786203</v>
       </c>
       <c r="F94">
         <v>0</v>
@@ -5357,7 +5357,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J94" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K94" t="str">
         <v>none</v>
@@ -5366,7 +5366,7 @@
         <v>0</v>
       </c>
       <c r="M94" t="str">
-        <v>2026-02-28T06:28:39.554Z</v>
+        <v>2026-07-05T04:07:08.327Z</v>
       </c>
       <c r="N94" t="str">
         <v/>
@@ -5383,19 +5383,19 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>Legacy</v>
+        <v>ad hoc</v>
       </c>
       <c r="B95">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C95">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D95">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E95">
-        <v>991.3908681786203</v>
+        <v>985</v>
       </c>
       <c r="F95">
         <v>0</v>
@@ -5410,7 +5410,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J95" t="str">
-        <v>AM</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K95" t="str">
         <v>none</v>
@@ -5419,7 +5419,7 @@
         <v>0</v>
       </c>
       <c r="M95" t="str">
-        <v>2026-07-05T04:07:08.327Z</v>
+        <v>2026-02-19T00:50:09.060Z</v>
       </c>
       <c r="N95" t="str">
         <v/>
@@ -5436,7 +5436,7 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>ad hoc</v>
+        <v>SAW</v>
       </c>
       <c r="B96">
         <v>0</v>
@@ -5463,7 +5463,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J96" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>EU</v>
       </c>
       <c r="K96" t="str">
         <v>none</v>
@@ -5472,7 +5472,7 @@
         <v>0</v>
       </c>
       <c r="M96" t="str">
-        <v>2026-02-19T00:50:09.060Z</v>
+        <v>2026-02-19T00:49:47.596Z</v>
       </c>
       <c r="N96" t="str">
         <v/>
@@ -5489,7 +5489,7 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>SAW</v>
+        <v>NomadS</v>
       </c>
       <c r="B97">
         <v>0</v>
@@ -5516,7 +5516,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J97" t="str">
-        <v>EU</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K97" t="str">
         <v>none</v>
@@ -5525,7 +5525,7 @@
         <v>0</v>
       </c>
       <c r="M97" t="str">
-        <v>2026-02-19T00:49:47.596Z</v>
+        <v>2026-02-19T00:49:35.489Z</v>
       </c>
       <c r="N97" t="str">
         <v/>
@@ -5542,7 +5542,7 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>NomadS</v>
+        <v>Outsiders</v>
       </c>
       <c r="B98">
         <v>0</v>
@@ -5569,7 +5569,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J98" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>EU</v>
       </c>
       <c r="K98" t="str">
         <v>none</v>
@@ -5578,7 +5578,7 @@
         <v>0</v>
       </c>
       <c r="M98" t="str">
-        <v>2026-02-19T00:49:35.489Z</v>
+        <v>2026-02-19T00:49:27.811Z</v>
       </c>
       <c r="N98" t="str">
         <v/>
@@ -5595,7 +5595,7 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Outsiders</v>
+        <v>Red Viperz</v>
       </c>
       <c r="B99">
         <v>0</v>
@@ -5622,7 +5622,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J99" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K99" t="str">
         <v>none</v>
@@ -5631,7 +5631,7 @@
         <v>0</v>
       </c>
       <c r="M99" t="str">
-        <v>2026-02-19T00:49:27.811Z</v>
+        <v>2026-02-19T00:49:20.687Z</v>
       </c>
       <c r="N99" t="str">
         <v/>
@@ -5648,7 +5648,7 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Red Viperz</v>
+        <v>The Dice</v>
       </c>
       <c r="B100">
         <v>0</v>
@@ -5675,7 +5675,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J100" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K100" t="str">
         <v>none</v>
@@ -5684,7 +5684,7 @@
         <v>0</v>
       </c>
       <c r="M100" t="str">
-        <v>2026-02-19T00:49:20.687Z</v>
+        <v>2026-02-19T00:49:12.765Z</v>
       </c>
       <c r="N100" t="str">
         <v/>
@@ -5701,7 +5701,7 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>The Dice</v>
+        <v>Victores Sumus</v>
       </c>
       <c r="B101">
         <v>0</v>
@@ -5728,7 +5728,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J101" t="str">
-        <v>EU</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K101" t="str">
         <v>none</v>
@@ -5737,7 +5737,7 @@
         <v>0</v>
       </c>
       <c r="M101" t="str">
-        <v>2026-02-19T00:49:12.765Z</v>
+        <v>2026-02-19T00:49:00.243Z</v>
       </c>
       <c r="N101" t="str">
         <v/>
@@ -5754,7 +5754,7 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>Victores Sumus</v>
+        <v>ODDIK</v>
       </c>
       <c r="B102">
         <v>0</v>
@@ -5781,7 +5781,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J102" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>AM</v>
       </c>
       <c r="K102" t="str">
         <v>none</v>
@@ -5790,7 +5790,7 @@
         <v>0</v>
       </c>
       <c r="M102" t="str">
-        <v>2026-02-19T00:49:00.243Z</v>
+        <v>2026-02-19T00:48:52.026Z</v>
       </c>
       <c r="N102" t="str">
         <v/>
@@ -5807,7 +5807,7 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>ODDIK</v>
+        <v>Qiang</v>
       </c>
       <c r="B103">
         <v>0</v>
@@ -5834,7 +5834,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J103" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K103" t="str">
         <v>none</v>
@@ -5843,7 +5843,7 @@
         <v>0</v>
       </c>
       <c r="M103" t="str">
-        <v>2026-02-19T00:48:52.026Z</v>
+        <v>2026-02-19T00:48:45.055Z</v>
       </c>
       <c r="N103" t="str">
         <v/>
@@ -5860,7 +5860,7 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>Qiang</v>
+        <v>inSanitY</v>
       </c>
       <c r="B104">
         <v>0</v>
@@ -5896,7 +5896,7 @@
         <v>0</v>
       </c>
       <c r="M104" t="str">
-        <v>2026-02-19T00:48:45.055Z</v>
+        <v>2026-02-19T00:48:38.129Z</v>
       </c>
       <c r="N104" t="str">
         <v/>
@@ -5913,7 +5913,7 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>inSanitY</v>
+        <v>Sangal</v>
       </c>
       <c r="B105">
         <v>0</v>
@@ -5949,7 +5949,7 @@
         <v>0</v>
       </c>
       <c r="M105" t="str">
-        <v>2026-02-19T00:48:38.129Z</v>
+        <v>2026-02-19T00:48:28.102Z</v>
       </c>
       <c r="N105" t="str">
         <v/>
@@ -5966,7 +5966,7 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>Sangal</v>
+        <v>9Pandas</v>
       </c>
       <c r="B106">
         <v>0</v>
@@ -6002,7 +6002,7 @@
         <v>0</v>
       </c>
       <c r="M106" t="str">
-        <v>2026-02-19T00:48:28.102Z</v>
+        <v>2026-02-19T00:48:17.012Z</v>
       </c>
       <c r="N106" t="str">
         <v/>
@@ -6019,7 +6019,7 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>9Pandas</v>
+        <v>Gods Reign</v>
       </c>
       <c r="B107">
         <v>0</v>
@@ -6055,7 +6055,7 @@
         <v>0</v>
       </c>
       <c r="M107" t="str">
-        <v>2026-02-19T00:48:17.012Z</v>
+        <v>2026-02-19T00:48:09.473Z</v>
       </c>
       <c r="N107" t="str">
         <v/>
@@ -6072,7 +6072,7 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>Gods Reign</v>
+        <v>CatEvil</v>
       </c>
       <c r="B108">
         <v>0</v>
@@ -6108,7 +6108,7 @@
         <v>0</v>
       </c>
       <c r="M108" t="str">
-        <v>2026-02-19T00:48:09.473Z</v>
+        <v>2026-02-19T00:48:02.110Z</v>
       </c>
       <c r="N108" t="str">
         <v/>
@@ -6125,7 +6125,7 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>CatEvil</v>
+        <v>Carnival</v>
       </c>
       <c r="B109">
         <v>0</v>
@@ -6161,7 +6161,7 @@
         <v>0</v>
       </c>
       <c r="M109" t="str">
-        <v>2026-02-19T00:48:02.110Z</v>
+        <v>2026-02-19T00:47:49.161Z</v>
       </c>
       <c r="N109" t="str">
         <v/>
@@ -6178,7 +6178,7 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>Carnival</v>
+        <v>Evil Geniuses</v>
       </c>
       <c r="B110">
         <v>0</v>
@@ -6214,7 +6214,7 @@
         <v>0</v>
       </c>
       <c r="M110" t="str">
-        <v>2026-02-19T00:47:49.161Z</v>
+        <v>2026-02-19T00:47:36.482Z</v>
       </c>
       <c r="N110" t="str">
         <v/>
@@ -6231,7 +6231,7 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>Evil Geniuses</v>
+        <v>Vantage</v>
       </c>
       <c r="B111">
         <v>0</v>
@@ -6267,7 +6267,7 @@
         <v>0</v>
       </c>
       <c r="M111" t="str">
-        <v>2026-02-19T00:47:36.482Z</v>
+        <v>2026-02-19T00:47:28.286Z</v>
       </c>
       <c r="N111" t="str">
         <v/>
@@ -6284,7 +6284,7 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>Vantage</v>
+        <v>ATOX</v>
       </c>
       <c r="B112">
         <v>0</v>
@@ -6311,7 +6311,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J112" t="str">
-        <v>EU</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K112" t="str">
         <v>none</v>
@@ -6320,7 +6320,7 @@
         <v>0</v>
       </c>
       <c r="M112" t="str">
-        <v>2026-02-19T00:47:28.286Z</v>
+        <v>2026-02-19T00:47:18.470Z</v>
       </c>
       <c r="N112" t="str">
         <v/>
@@ -6337,7 +6337,7 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>ATOX</v>
+        <v>Skinvault</v>
       </c>
       <c r="B113">
         <v>0</v>
@@ -6364,7 +6364,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J113" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>EU</v>
       </c>
       <c r="K113" t="str">
         <v>none</v>
@@ -6373,7 +6373,7 @@
         <v>0</v>
       </c>
       <c r="M113" t="str">
-        <v>2026-02-19T00:47:18.470Z</v>
+        <v>2026-02-19T00:47:11.265Z</v>
       </c>
       <c r="N113" t="str">
         <v/>
@@ -6390,7 +6390,7 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>Skinvault</v>
+        <v>BC.Game</v>
       </c>
       <c r="B114">
         <v>0</v>
@@ -6426,7 +6426,7 @@
         <v>0</v>
       </c>
       <c r="M114" t="str">
-        <v>2026-02-19T00:47:11.265Z</v>
+        <v>2026-02-19T00:46:52.846Z</v>
       </c>
       <c r="N114" t="str">
         <v/>
@@ -6443,7 +6443,7 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>BC.Game</v>
+        <v>Wings Up</v>
       </c>
       <c r="B115">
         <v>0</v>
@@ -6470,7 +6470,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J115" t="str">
-        <v>EU</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K115" t="str">
         <v>none</v>
@@ -6479,7 +6479,7 @@
         <v>0</v>
       </c>
       <c r="M115" t="str">
-        <v>2026-02-19T00:46:52.846Z</v>
+        <v>2026-02-19T00:46:32.115Z</v>
       </c>
       <c r="N115" t="str">
         <v/>
@@ -6496,7 +6496,7 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>Wings Up</v>
+        <v>Lynn Vision</v>
       </c>
       <c r="B116">
         <v>0</v>
@@ -6532,7 +6532,7 @@
         <v>0</v>
       </c>
       <c r="M116" t="str">
-        <v>2026-02-19T00:46:32.115Z</v>
+        <v>2026-02-19T00:46:08.336Z</v>
       </c>
       <c r="N116" t="str">
         <v/>
@@ -6549,7 +6549,7 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>Lynn Vision</v>
+        <v>Tricked</v>
       </c>
       <c r="B117">
         <v>0</v>
@@ -6576,7 +6576,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J117" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>EU</v>
       </c>
       <c r="K117" t="str">
         <v>none</v>
@@ -6585,7 +6585,7 @@
         <v>0</v>
       </c>
       <c r="M117" t="str">
-        <v>2026-02-19T00:46:08.336Z</v>
+        <v>2026-02-19T00:45:42.234Z</v>
       </c>
       <c r="N117" t="str">
         <v/>
@@ -6602,7 +6602,7 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>Tricked</v>
+        <v>3DMAX</v>
       </c>
       <c r="B118">
         <v>0</v>
@@ -6638,7 +6638,7 @@
         <v>0</v>
       </c>
       <c r="M118" t="str">
-        <v>2026-02-19T00:45:42.234Z</v>
+        <v>2026-02-19T00:39:02.710Z</v>
       </c>
       <c r="N118" t="str">
         <v/>
@@ -6655,7 +6655,7 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>3DMAX</v>
+        <v>Venom</v>
       </c>
       <c r="B119">
         <v>0</v>
@@ -6682,7 +6682,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J119" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K119" t="str">
         <v>none</v>
@@ -6691,7 +6691,7 @@
         <v>0</v>
       </c>
       <c r="M119" t="str">
-        <v>2026-02-19T00:39:02.710Z</v>
+        <v>2026-02-19T00:38:39.010Z</v>
       </c>
       <c r="N119" t="str">
         <v/>
@@ -6708,7 +6708,7 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>Venom</v>
+        <v>ARCRED</v>
       </c>
       <c r="B120">
         <v>0</v>
@@ -6735,7 +6735,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J120" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K120" t="str">
         <v>none</v>
@@ -6744,7 +6744,7 @@
         <v>0</v>
       </c>
       <c r="M120" t="str">
-        <v>2026-02-19T00:38:39.010Z</v>
+        <v>2026-02-19T00:38:03.598Z</v>
       </c>
       <c r="N120" t="str">
         <v/>
@@ -6761,7 +6761,7 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>ARCRED</v>
+        <v>GamerLegion</v>
       </c>
       <c r="B121">
         <v>0</v>
@@ -6788,7 +6788,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J121" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K121" t="str">
         <v>none</v>
@@ -6797,7 +6797,7 @@
         <v>0</v>
       </c>
       <c r="M121" t="str">
-        <v>2026-02-19T00:38:03.598Z</v>
+        <v>2026-02-19T00:37:47.172Z</v>
       </c>
       <c r="N121" t="str">
         <v/>
@@ -6814,7 +6814,7 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>GamerLegion</v>
+        <v>Passion UA</v>
       </c>
       <c r="B122">
         <v>0</v>
@@ -6841,7 +6841,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J122" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K122" t="str">
         <v>none</v>
@@ -6850,7 +6850,7 @@
         <v>0</v>
       </c>
       <c r="M122" t="str">
-        <v>2026-02-19T00:37:47.172Z</v>
+        <v>2026-02-19T00:37:27.234Z</v>
       </c>
       <c r="N122" t="str">
         <v/>
@@ -6867,7 +6867,7 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>Passion UA</v>
+        <v>FlyQuest</v>
       </c>
       <c r="B123">
         <v>0</v>
@@ -6894,7 +6894,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J123" t="str">
-        <v>EU</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K123" t="str">
         <v>none</v>
@@ -6903,7 +6903,7 @@
         <v>0</v>
       </c>
       <c r="M123" t="str">
-        <v>2026-02-19T00:37:27.234Z</v>
+        <v>2026-02-19T00:37:20.280Z</v>
       </c>
       <c r="N123" t="str">
         <v/>
@@ -6920,7 +6920,7 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>FlyQuest</v>
+        <v>Envy</v>
       </c>
       <c r="B124">
         <v>0</v>
@@ -6947,7 +6947,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J124" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>EU</v>
       </c>
       <c r="K124" t="str">
         <v>none</v>
@@ -6956,7 +6956,7 @@
         <v>0</v>
       </c>
       <c r="M124" t="str">
-        <v>2026-02-19T00:37:20.280Z</v>
+        <v>2026-02-19T00:37:05.560Z</v>
       </c>
       <c r="N124" t="str">
         <v/>
@@ -6973,7 +6973,7 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>Envy</v>
+        <v>BIG</v>
       </c>
       <c r="B125">
         <v>0</v>
@@ -7009,7 +7009,7 @@
         <v>0</v>
       </c>
       <c r="M125" t="str">
-        <v>2026-02-19T00:37:05.560Z</v>
+        <v>2026-02-19T00:36:43.463Z</v>
       </c>
       <c r="N125" t="str">
         <v/>
@@ -7026,7 +7026,7 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>BIG</v>
+        <v>Limitless</v>
       </c>
       <c r="B126">
         <v>0</v>
@@ -7062,7 +7062,7 @@
         <v>0</v>
       </c>
       <c r="M126" t="str">
-        <v>2026-02-19T00:36:43.463Z</v>
+        <v>2026-02-19T00:36:26.343Z</v>
       </c>
       <c r="N126" t="str">
         <v/>
@@ -7079,7 +7079,7 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>Limitless</v>
+        <v>Galorys</v>
       </c>
       <c r="B127">
         <v>0</v>
@@ -7106,7 +7106,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J127" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K127" t="str">
         <v>none</v>
@@ -7115,7 +7115,7 @@
         <v>0</v>
       </c>
       <c r="M127" t="str">
-        <v>2026-02-19T00:36:26.343Z</v>
+        <v>2026-02-19T00:36:18.696Z</v>
       </c>
       <c r="N127" t="str">
         <v/>
@@ -7132,7 +7132,7 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>Galorys</v>
+        <v>devils.one</v>
       </c>
       <c r="B128">
         <v>0</v>
@@ -7159,7 +7159,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J128" t="str">
-        <v>AM</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K128" t="str">
         <v>none</v>
@@ -7168,7 +7168,7 @@
         <v>0</v>
       </c>
       <c r="M128" t="str">
-        <v>2026-02-19T00:36:18.696Z</v>
+        <v>2026-02-18T21:23:30.347Z</v>
       </c>
       <c r="N128" t="str">
         <v/>
@@ -7185,7 +7185,7 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>devils.one</v>
+        <v>Luminosity</v>
       </c>
       <c r="B129">
         <v>0</v>
@@ -7212,7 +7212,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J129" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>EU</v>
       </c>
       <c r="K129" t="str">
         <v>none</v>
@@ -7221,7 +7221,7 @@
         <v>0</v>
       </c>
       <c r="M129" t="str">
-        <v>2026-02-18T21:23:30.347Z</v>
+        <v>2026-02-18T21:23:18.851Z</v>
       </c>
       <c r="N129" t="str">
         <v/>
@@ -7238,7 +7238,7 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>Luminosity</v>
+        <v>Sharks</v>
       </c>
       <c r="B130">
         <v>0</v>
@@ -7265,7 +7265,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J130" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K130" t="str">
         <v>none</v>
@@ -7274,7 +7274,7 @@
         <v>0</v>
       </c>
       <c r="M130" t="str">
-        <v>2026-02-18T21:23:18.851Z</v>
+        <v>2026-02-18T21:23:12.952Z</v>
       </c>
       <c r="N130" t="str">
         <v/>
@@ -7291,7 +7291,7 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>Sharks</v>
+        <v>IHC</v>
       </c>
       <c r="B131">
         <v>0</v>
@@ -7318,7 +7318,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J131" t="str">
-        <v>AM</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K131" t="str">
         <v>none</v>
@@ -7327,7 +7327,7 @@
         <v>0</v>
       </c>
       <c r="M131" t="str">
-        <v>2026-02-18T21:23:12.952Z</v>
+        <v>2026-02-18T21:23:06.529Z</v>
       </c>
       <c r="N131" t="str">
         <v/>
@@ -7344,7 +7344,7 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>IHC</v>
+        <v>Kappa Bar</v>
       </c>
       <c r="B132">
         <v>0</v>
@@ -7371,7 +7371,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J132" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>EU</v>
       </c>
       <c r="K132" t="str">
         <v>none</v>
@@ -7380,7 +7380,7 @@
         <v>0</v>
       </c>
       <c r="M132" t="str">
-        <v>2026-02-18T21:23:06.529Z</v>
+        <v>2026-02-18T21:22:57.244Z</v>
       </c>
       <c r="N132" t="str">
         <v/>
@@ -7397,7 +7397,7 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>Kappa Bar</v>
+        <v>Complexity</v>
       </c>
       <c r="B133">
         <v>0</v>
@@ -7424,7 +7424,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J133" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K133" t="str">
         <v>none</v>
@@ -7433,7 +7433,7 @@
         <v>0</v>
       </c>
       <c r="M133" t="str">
-        <v>2026-02-18T21:22:57.244Z</v>
+        <v>2026-02-18T21:22:48.652Z</v>
       </c>
       <c r="N133" t="str">
         <v/>
@@ -7450,7 +7450,7 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>Complexity</v>
+        <v>Case</v>
       </c>
       <c r="B134">
         <v>0</v>
@@ -7477,7 +7477,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J134" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K134" t="str">
         <v>none</v>
@@ -7486,7 +7486,7 @@
         <v>0</v>
       </c>
       <c r="M134" t="str">
-        <v>2026-02-18T21:22:48.652Z</v>
+        <v>2026-02-18T21:22:39.402Z</v>
       </c>
       <c r="N134" t="str">
         <v/>
@@ -7503,7 +7503,7 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>Case</v>
+        <v>Enemy</v>
       </c>
       <c r="B135">
         <v>0</v>
@@ -7539,7 +7539,7 @@
         <v>0</v>
       </c>
       <c r="M135" t="str">
-        <v>2026-02-18T21:22:39.402Z</v>
+        <v>2026-02-18T21:22:20.745Z</v>
       </c>
       <c r="N135" t="str">
         <v/>
@@ -7556,7 +7556,7 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>Enemy</v>
+        <v>KRU</v>
       </c>
       <c r="B136">
         <v>0</v>
@@ -7583,7 +7583,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J136" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K136" t="str">
         <v>none</v>
@@ -7592,7 +7592,7 @@
         <v>0</v>
       </c>
       <c r="M136" t="str">
-        <v>2026-02-18T21:22:20.745Z</v>
+        <v>2026-02-18T21:22:06.663Z</v>
       </c>
       <c r="N136" t="str">
         <v/>
@@ -7609,7 +7609,7 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>KRU</v>
+        <v>Imperial</v>
       </c>
       <c r="B137">
         <v>0</v>
@@ -7645,7 +7645,7 @@
         <v>0</v>
       </c>
       <c r="M137" t="str">
-        <v>2026-02-18T21:22:06.663Z</v>
+        <v>2026-02-18T21:21:57.658Z</v>
       </c>
       <c r="N137" t="str">
         <v/>
@@ -7662,7 +7662,7 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>Imperial</v>
+        <v>paiN</v>
       </c>
       <c r="B138">
         <v>0</v>
@@ -7698,7 +7698,7 @@
         <v>0</v>
       </c>
       <c r="M138" t="str">
-        <v>2026-02-18T21:21:57.658Z</v>
+        <v>2026-02-18T21:21:14.058Z</v>
       </c>
       <c r="N138" t="str">
         <v/>
@@ -7715,7 +7715,7 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>paiN</v>
+        <v>Vexed</v>
       </c>
       <c r="B139">
         <v>0</v>
@@ -7742,7 +7742,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J139" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K139" t="str">
         <v>none</v>
@@ -7751,7 +7751,7 @@
         <v>0</v>
       </c>
       <c r="M139" t="str">
-        <v>2026-02-18T21:21:14.058Z</v>
+        <v>2026-02-18T21:19:58.722Z</v>
       </c>
       <c r="N139" t="str">
         <v/>
@@ -7768,19 +7768,19 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>Vexed</v>
+        <v>Dignitas</v>
       </c>
       <c r="B140">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C140">
         <v>0</v>
       </c>
       <c r="D140">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E140">
-        <v>985</v>
+        <v>984.7039370196626</v>
       </c>
       <c r="F140">
         <v>0</v>
@@ -7804,7 +7804,7 @@
         <v>0</v>
       </c>
       <c r="M140" t="str">
-        <v>2026-02-18T21:19:58.722Z</v>
+        <v>2026-02-19T21:54:17.535Z</v>
       </c>
       <c r="N140" t="str">
         <v/>
@@ -7821,7 +7821,7 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>Dignitas</v>
+        <v>LDLC</v>
       </c>
       <c r="B141">
         <v>1</v>
@@ -7857,7 +7857,7 @@
         <v>0</v>
       </c>
       <c r="M141" t="str">
-        <v>2026-02-19T21:54:17.535Z</v>
+        <v>2026-02-19T21:53:53.691Z</v>
       </c>
       <c r="N141" t="str">
         <v/>
@@ -7874,7 +7874,7 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>LDLC</v>
+        <v>Aravt</v>
       </c>
       <c r="B142">
         <v>1</v>
@@ -7910,7 +7910,7 @@
         <v>0</v>
       </c>
       <c r="M142" t="str">
-        <v>2026-02-19T21:53:53.691Z</v>
+        <v>2026-02-19T02:51:09.872Z</v>
       </c>
       <c r="N142" t="str">
         <v/>
@@ -7927,7 +7927,7 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>Aravt</v>
+        <v>VP.Prodigy</v>
       </c>
       <c r="B143">
         <v>1</v>
@@ -7963,7 +7963,7 @@
         <v>0</v>
       </c>
       <c r="M143" t="str">
-        <v>2026-02-19T02:51:09.872Z</v>
+        <v>2026-02-19T02:51:03.784Z</v>
       </c>
       <c r="N143" t="str">
         <v/>
@@ -7980,7 +7980,7 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>VP.Prodigy</v>
+        <v>Underground</v>
       </c>
       <c r="B144">
         <v>1</v>
@@ -8016,7 +8016,7 @@
         <v>0</v>
       </c>
       <c r="M144" t="str">
-        <v>2026-02-19T02:51:03.784Z</v>
+        <v>2026-02-19T02:47:27.422Z</v>
       </c>
       <c r="N144" t="str">
         <v/>
@@ -8033,7 +8033,7 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>Entropiq</v>
+        <v>Virtus.pro</v>
       </c>
       <c r="B145">
         <v>1</v>
@@ -8060,7 +8060,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J145" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K145" t="str">
         <v>none</v>
@@ -8069,7 +8069,7 @@
         <v>0</v>
       </c>
       <c r="M145" t="str">
-        <v>2026-02-19T02:49:25.044Z</v>
+        <v>2026-02-19T02:47:19.575Z</v>
       </c>
       <c r="N145" t="str">
         <v/>
@@ -8086,7 +8086,7 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>Underground</v>
+        <v>ShindeN</v>
       </c>
       <c r="B146">
         <v>1</v>
@@ -8122,7 +8122,7 @@
         <v>0</v>
       </c>
       <c r="M146" t="str">
-        <v>2026-02-19T02:47:27.422Z</v>
+        <v>2026-02-19T02:36:26.535Z</v>
       </c>
       <c r="N146" t="str">
         <v/>
@@ -8139,7 +8139,7 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>Virtus.pro</v>
+        <v>Permitta</v>
       </c>
       <c r="B147">
         <v>1</v>
@@ -8175,7 +8175,7 @@
         <v>0</v>
       </c>
       <c r="M147" t="str">
-        <v>2026-02-19T02:47:19.575Z</v>
+        <v>2026-02-19T02:36:17.329Z</v>
       </c>
       <c r="N147" t="str">
         <v/>
@@ -8192,7 +8192,7 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>ShindeN</v>
+        <v>Wildcard</v>
       </c>
       <c r="B148">
         <v>1</v>
@@ -8219,7 +8219,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J148" t="str">
-        <v>EU</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K148" t="str">
         <v>none</v>
@@ -8228,7 +8228,7 @@
         <v>0</v>
       </c>
       <c r="M148" t="str">
-        <v>2026-02-19T02:36:26.535Z</v>
+        <v>2026-02-19T02:34:08.116Z</v>
       </c>
       <c r="N148" t="str">
         <v/>
@@ -8245,7 +8245,7 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>Permitta</v>
+        <v>Astralis</v>
       </c>
       <c r="B149">
         <v>1</v>
@@ -8281,7 +8281,7 @@
         <v>0</v>
       </c>
       <c r="M149" t="str">
-        <v>2026-02-19T02:36:17.329Z</v>
+        <v>2026-02-19T02:34:01.822Z</v>
       </c>
       <c r="N149" t="str">
         <v/>
@@ -8298,7 +8298,7 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>Wildcard</v>
+        <v>Bad News Eagles</v>
       </c>
       <c r="B150">
         <v>1</v>
@@ -8325,7 +8325,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J150" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>AM</v>
       </c>
       <c r="K150" t="str">
         <v>none</v>
@@ -8334,7 +8334,7 @@
         <v>0</v>
       </c>
       <c r="M150" t="str">
-        <v>2026-02-19T02:34:08.116Z</v>
+        <v>2026-02-19T01:45:27.335Z</v>
       </c>
       <c r="N150" t="str">
         <v/>
@@ -8351,7 +8351,7 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>Astralis</v>
+        <v>SK</v>
       </c>
       <c r="B151">
         <v>1</v>
@@ -8378,7 +8378,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J151" t="str">
-        <v>EU</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K151" t="str">
         <v>none</v>
@@ -8387,7 +8387,7 @@
         <v>0</v>
       </c>
       <c r="M151" t="str">
-        <v>2026-02-19T02:34:01.822Z</v>
+        <v>2026-02-19T01:39:18.535Z</v>
       </c>
       <c r="N151" t="str">
         <v/>
@@ -8404,7 +8404,7 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>Bad News Eagles</v>
+        <v>ECSTATIC</v>
       </c>
       <c r="B152">
         <v>1</v>
@@ -8431,7 +8431,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J152" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K152" t="str">
         <v>none</v>
@@ -8440,7 +8440,7 @@
         <v>0</v>
       </c>
       <c r="M152" t="str">
-        <v>2026-02-19T01:45:27.335Z</v>
+        <v>2026-02-19T01:39:12.540Z</v>
       </c>
       <c r="N152" t="str">
         <v/>
@@ -8457,7 +8457,7 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>SK</v>
+        <v>MIBR Academy</v>
       </c>
       <c r="B153">
         <v>1</v>
@@ -8469,7 +8469,7 @@
         <v>2</v>
       </c>
       <c r="E153">
-        <v>984.7039370196626</v>
+        <v>984.075576101157</v>
       </c>
       <c r="F153">
         <v>0</v>
@@ -8484,7 +8484,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J153" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>AM</v>
       </c>
       <c r="K153" t="str">
         <v>none</v>
@@ -8493,7 +8493,7 @@
         <v>0</v>
       </c>
       <c r="M153" t="str">
-        <v>2026-02-19T01:39:18.535Z</v>
+        <v>2026-06-26T13:19:31.639Z</v>
       </c>
       <c r="N153" t="str">
         <v/>
@@ -8510,7 +8510,7 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>ECSTATIC</v>
+        <v>paiN Academy</v>
       </c>
       <c r="B154">
         <v>1</v>
@@ -8522,7 +8522,7 @@
         <v>2</v>
       </c>
       <c r="E154">
-        <v>984.7039370196626</v>
+        <v>984.0732769617838</v>
       </c>
       <c r="F154">
         <v>0</v>
@@ -8537,7 +8537,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J154" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K154" t="str">
         <v>none</v>
@@ -8546,7 +8546,7 @@
         <v>0</v>
       </c>
       <c r="M154" t="str">
-        <v>2026-02-19T01:39:12.540Z</v>
+        <v>2026-07-07T04:08:50.601Z</v>
       </c>
       <c r="N154" t="str">
         <v/>
@@ -8563,19 +8563,19 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>MIBR Academy</v>
+        <v>TALON</v>
       </c>
       <c r="B155">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C155">
         <v>0</v>
       </c>
       <c r="D155">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E155">
-        <v>984.075576101157</v>
+        <v>983.9905713816794</v>
       </c>
       <c r="F155">
         <v>0</v>
@@ -8590,7 +8590,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J155" t="str">
-        <v>AM</v>
+        <v>AS/SIS/ESEA</v>
       </c>
       <c r="K155" t="str">
         <v>none</v>
@@ -8599,7 +8599,7 @@
         <v>0</v>
       </c>
       <c r="M155" t="str">
-        <v>2026-06-26T13:19:31.639Z</v>
+        <v>2026-02-28T06:27:14.538Z</v>
       </c>
       <c r="N155" t="str">
         <v/>
@@ -8616,19 +8616,19 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>TALON</v>
+        <v>B8</v>
       </c>
       <c r="B156">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C156">
         <v>0</v>
       </c>
       <c r="D156">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E156">
-        <v>983.9905713816794</v>
+        <v>983.4284201175154</v>
       </c>
       <c r="F156">
         <v>0</v>
@@ -8643,7 +8643,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J156" t="str">
-        <v>AS/SIS/ESEA</v>
+        <v>AM</v>
       </c>
       <c r="K156" t="str">
         <v>none</v>
@@ -8652,7 +8652,7 @@
         <v>0</v>
       </c>
       <c r="M156" t="str">
-        <v>2026-02-28T06:27:14.538Z</v>
+        <v>2026-07-05T04:05:49.346Z</v>
       </c>
       <c r="N156" t="str">
         <v/>
@@ -8669,19 +8669,19 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>B8</v>
+        <v>NAVI Junior</v>
       </c>
       <c r="B157">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C157">
         <v>0</v>
       </c>
       <c r="D157">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E157">
-        <v>983.4284201175154</v>
+        <v>983.2698348870488</v>
       </c>
       <c r="F157">
         <v>0</v>
@@ -8696,7 +8696,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J157" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K157" t="str">
         <v>none</v>
@@ -8705,7 +8705,7 @@
         <v>0</v>
       </c>
       <c r="M157" t="str">
-        <v>2026-07-05T04:05:49.346Z</v>
+        <v>2026-02-28T06:27:03.939Z</v>
       </c>
       <c r="N157" t="str">
         <v/>
@@ -8722,19 +8722,19 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>NAVI Junior</v>
+        <v>9z</v>
       </c>
       <c r="B158">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C158">
         <v>0</v>
       </c>
       <c r="D158">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E158">
-        <v>983.2698348870488</v>
+        <v>971.3809496889581</v>
       </c>
       <c r="F158">
         <v>0</v>
@@ -8749,7 +8749,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J158" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K158" t="str">
         <v>none</v>
@@ -8758,7 +8758,7 @@
         <v>0</v>
       </c>
       <c r="M158" t="str">
-        <v>2026-02-28T06:27:03.939Z</v>
+        <v>2026-07-05T04:07:15.376Z</v>
       </c>
       <c r="N158" t="str">
         <v/>
@@ -8775,19 +8775,19 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>9z</v>
+        <v>Ninjas in Pyjamas</v>
       </c>
       <c r="B159">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C159">
         <v>0</v>
       </c>
       <c r="D159">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E159">
-        <v>971.3809496889581</v>
+        <v>970</v>
       </c>
       <c r="F159">
         <v>0</v>
@@ -8802,7 +8802,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J159" t="str">
-        <v>AM</v>
+        <v>EU</v>
       </c>
       <c r="K159" t="str">
         <v>none</v>
@@ -8811,7 +8811,7 @@
         <v>0</v>
       </c>
       <c r="M159" t="str">
-        <v>2026-07-05T04:07:15.376Z</v>
+        <v>2026-02-19T21:53:46.615Z</v>
       </c>
       <c r="N159" t="str">
         <v/>
@@ -8828,7 +8828,7 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>Ninjas in Pyjamas</v>
+        <v>MOUZ</v>
       </c>
       <c r="B160">
         <v>0</v>
@@ -8864,7 +8864,7 @@
         <v>0</v>
       </c>
       <c r="M160" t="str">
-        <v>2026-02-19T21:53:46.615Z</v>
+        <v>2026-02-19T21:53:40.004Z</v>
       </c>
       <c r="N160" t="str">
         <v/>
@@ -8881,7 +8881,7 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>MOUZ</v>
+        <v>Aurora</v>
       </c>
       <c r="B161">
         <v>0</v>
@@ -8917,7 +8917,7 @@
         <v>0</v>
       </c>
       <c r="M161" t="str">
-        <v>2026-02-19T21:53:40.004Z</v>
+        <v>2026-02-19T21:53:30.387Z</v>
       </c>
       <c r="N161" t="str">
         <v/>
@@ -8934,7 +8934,7 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>Aurora</v>
+        <v>Reason</v>
       </c>
       <c r="B162">
         <v>0</v>
@@ -8970,7 +8970,7 @@
         <v>0</v>
       </c>
       <c r="M162" t="str">
-        <v>2026-02-19T21:53:30.387Z</v>
+        <v>2026-02-19T21:53:23.315Z</v>
       </c>
       <c r="N162" t="str">
         <v/>
@@ -8987,7 +8987,7 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>Reason</v>
+        <v>Sprout</v>
       </c>
       <c r="B163">
         <v>0</v>
@@ -8999,7 +8999,7 @@
         <v>2</v>
       </c>
       <c r="E163">
-        <v>970</v>
+        <v>969.9715073660867</v>
       </c>
       <c r="F163">
         <v>0</v>
@@ -9014,7 +9014,7 @@
         <v>Tier 3</v>
       </c>
       <c r="J163" t="str">
-        <v>EU</v>
+        <v>AM</v>
       </c>
       <c r="K163" t="str">
         <v>none</v>
@@ -9023,7 +9023,7 @@
         <v>0</v>
       </c>
       <c r="M163" t="str">
-        <v>2026-02-19T21:53:23.315Z</v>
+        <v>2026-07-07T04:07:21.355Z</v>
       </c>
       <c r="N163" t="str">
         <v/>

</xml_diff>